<commit_message>
Deploying to gh-pages from @ eurovibes/sertest-ng@d87ae5931d802483cd956921e99df2dbb285ed76 🚀
</commit_message>
<xml_diff>
--- a/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
+++ b/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
@@ -170,7 +170,7 @@
     <t>D201 D202 D203 D204 D205 D206 D207 D208 D209 D210 D211 D212 D213 D214 D401 D402</t>
   </si>
   <si>
-    <t>LED_Dual_AAKK</t>
+    <t>LED_Dual_KAAK</t>
   </si>
   <si>
     <t>RI</t>
@@ -182,7 +182,7 @@
     <t>LED_Kingbright_AAA3528ESGCT</t>
   </si>
   <si>
-    <t>Dual LED, cathodes on pins 3 and 4</t>
+    <t>Dual LED, cathodes on pins 1 and 4</t>
   </si>
   <si>
     <t>16</t>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ eurovibes/sertest-ng@fd12f7b8a575bdaec5f4aed8c1687597aec7e080 🚀
</commit_message>
<xml_diff>
--- a/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
+++ b/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
@@ -59,13 +59,13 @@
     <t>1</t>
   </si>
   <si>
-    <t>C101 C102 C103 C104 C105 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C201 C202 C203 C204 C205 C206 C207 C208 C301 C302 C303 C304 C401</t>
+    <t>C101 C102 C103 C104 C106 C107 C108 C109 C110 C111 C112 C113 C114 C115 C116 C201 C202 C203 C204 C205 C206 C207 C208 C301 C302 C303 C304 C401</t>
   </si>
   <si>
     <t>C</t>
   </si>
   <si>
-    <t>100 nF</t>
+    <t>20 pF</t>
   </si>
   <si>
     <t>CL05B104KB54PNC CL10A105KB8NNNC 0402B472K500NT</t>
@@ -80,7 +80,7 @@
     <t/>
   </si>
   <si>
-    <t>https://jlcpcb.com/partdetail/291005-CL05B104KB54PNC/C307331 https://jlcpcb.com/partdetail/1906-0402CG200J500NT/C1554 https://jlcpcb.com/partdetail/16532-CL21A106KAYNNNE/C15850 https://jlcpcb.com/partdetail/1899-0402CG120J500NT/C1547 https://jlcpcb.com/partdetail/16531-CL10A105KB8NNNC/C15849 https://jlcpcb.com/partdetail/1890-0402B472K500NT/C1538</t>
+    <t>https://jlcpcb.com/partdetail/1906-0402CG200J500NT/C1554 https://jlcpcb.com/partdetail/1899-0402CG120J500NT/C1547 https://jlcpcb.com/partdetail/291005-CL05B104KB54PNC/C307331 https://jlcpcb.com/partdetail/16532-CL21A106KAYNNNE/C15850 https://jlcpcb.com/partdetail/16531-CL10A105KB8NNNC/C15849 https://jlcpcb.com/partdetail/1890-0402B472K500NT/C1538</t>
   </si>
   <si>
     <t>C_0402_1005Metric</t>
@@ -95,7 +95,7 @@
     <t>2</t>
   </si>
   <si>
-    <t>C106</t>
+    <t>C105</t>
   </si>
   <si>
     <t>C_Polarized</t>
@@ -266,7 +266,7 @@
     <t>10</t>
   </si>
   <si>
-    <t>J102 J301</t>
+    <t>J101 J301</t>
   </si>
   <si>
     <t>USB_C_Receptacle_USB2.0_16P</t>
@@ -287,7 +287,7 @@
     <t>11</t>
   </si>
   <si>
-    <t>JP403</t>
+    <t>JP401</t>
   </si>
   <si>
     <t>Jumper_2_Open</t>
@@ -305,7 +305,7 @@
     <t>12</t>
   </si>
   <si>
-    <t>R406 R408</t>
+    <t>R405 R406</t>
   </si>
   <si>
     <t>R</t>
@@ -332,7 +332,7 @@
     <t>13</t>
   </si>
   <si>
-    <t>R405 R407</t>
+    <t>R407 R408</t>
   </si>
   <si>
     <t>100 Ω</t>
@@ -350,7 +350,7 @@
     <t>14</t>
   </si>
   <si>
-    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R201 R202 R203 R204 R205 R206 R207 R208 R209 R210 R211 R212 R213 R214 R215 R216 R217 R218 R219 R220 R221 R222 R223 R224 R225 R226 R227 R228 R229 R230 R231 R232 R301 R302 R303 R401 R402 R403 R404</t>
+    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R201 R202 R203 R204 R205 R206 R207 R208 R209 R210 R211 R212 R213 R214 R215 R216 R217 R218 R219 R220 R221 R222 R223 R224 R225 R226 R227 R228 R229 R230 R231 R232 R301 R302 R303 R401 R402 R403 R404</t>
   </si>
   <si>
     <t>1 kΩ</t>
@@ -359,10 +359,10 @@
     <t>0402WGF1001TCE</t>
   </si>
   <si>
-    <t>https://jlcpcb.com/partdetail/12256-0402WGF1001TCE/C11702 https://jlcpcb.com/partdetail/18646-1206W4F220JT5E/C17958 https://jlcpcb.com/partdetail/26826-0402WGF1004TCE/C26083 https://jlcpcb.com/partdetail/26648-0402WGF5101TCE/C25905 https://jlcpcb.com/partdetail/17853-0402WGF0000TCE/C17168</t>
-  </si>
-  <si>
-    <t>51</t>
+    <t>https://jlcpcb.com/partdetail/12256-0402WGF1001TCE/C11702 https://jlcpcb.com/partdetail/26648-0402WGF5101TCE/C25905 https://jlcpcb.com/partdetail/26826-0402WGF1004TCE/C26083 https://jlcpcb.com/partdetail/18646-1206W4F220JT5E/C17958 https://jlcpcb.com/partdetail/25848-0402WGF330JTCE/C25105 https://jlcpcb.com/partdetail/26487-0402WGF1002TCE/C25744 https://jlcpcb.com/partdetail/17853-0402WGF0000TCE/C17168</t>
+  </si>
+  <si>
+    <t>54</t>
   </si>
   <si>
     <t>15</t>
@@ -434,7 +434,7 @@
     <t>18</t>
   </si>
   <si>
-    <t>U102</t>
+    <t>U105</t>
   </si>
   <si>
     <t>AMS1117-3.3</t>
@@ -476,127 +476,127 @@
     <t>20</t>
   </si>
   <si>
+    <t>U303</t>
+  </si>
+  <si>
+    <t>CH340N</t>
+  </si>
+  <si>
+    <t>WCH(Jiangsu Qin Heng)</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/TorexSemicon-XC6206P332MRG/C5446</t>
+  </si>
+  <si>
+    <t>JEITA_SOIC-8_3.9x4.9mm_P1.27mm</t>
+  </si>
+  <si>
+    <t>USB serial converter, 2Mbps, UART, JEITA SOIC-8 (SOP-8)</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>U101</t>
+  </si>
+  <si>
+    <t>M24C02-RMN</t>
+  </si>
+  <si>
+    <t>M24C64-RMN</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/STMicroelectronics-M24C64RMN6TP/C79988</t>
+  </si>
+  <si>
+    <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+  </si>
+  <si>
+    <t>2Kb (256x8) I2C Serial EEPROM, 1.8-5.5V, SOIC-8</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>U202</t>
+  </si>
+  <si>
+    <t>SP330</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/MaxLinear-SP330EEY_LTR/C916084</t>
+  </si>
+  <si>
+    <t>TSSOP-24_4.4x7.8mm_P0.65mm</t>
+  </si>
+  <si>
+    <t>RS-232/RS-485/RS-422 Transceiver with 1.65V-5.5V Interface</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>U103</t>
+  </si>
+  <si>
+    <t>STM32G431RBTx</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/STMicroelectronics-STM32G431RBT6/C431633</t>
+  </si>
+  <si>
+    <t>LQFP-64_10x10mm_P0.5mm</t>
+  </si>
+  <si>
+    <t>STMicroelectronics Arm Cortex-M4 MCU, 128KB flash, 32KB RAM, 170 MHz, 1.71-3.6V, 52 GPIO, LQFP64</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>U401</t>
+  </si>
+  <si>
+    <t>TJA1042T</t>
+  </si>
+  <si>
+    <t>TJA1042T/1J</t>
+  </si>
+  <si>
+    <t>NXP Semicon</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/NXPSemicon-TJA1042T1J/C53670</t>
+  </si>
+  <si>
+    <t>High-Speed CAN Transceiver, standby mode, split pin, SOIC-8</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>U102 U301</t>
+  </si>
+  <si>
+    <t>USBLC6-2SC6</t>
+  </si>
+  <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/partdetail/2790619-USBLC62SC6/C2687116</t>
+  </si>
+  <si>
+    <t>SOT-23-6</t>
+  </si>
+  <si>
+    <t>Very low capacitance ESD protection diode, 2 data-line, SOT-23-6</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
     <t>U302</t>
-  </si>
-  <si>
-    <t>CH340N</t>
-  </si>
-  <si>
-    <t>WCH(Jiangsu Qin Heng)</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/TorexSemicon-XC6206P332MRG/C5446</t>
-  </si>
-  <si>
-    <t>JEITA_SOIC-8_3.9x4.9mm_P1.27mm</t>
-  </si>
-  <si>
-    <t>USB serial converter, 2Mbps, UART, JEITA SOIC-8 (SOP-8)</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>U101</t>
-  </si>
-  <si>
-    <t>M24C02-RMN</t>
-  </si>
-  <si>
-    <t>M24C64-RMN</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/STMicroelectronics-M24C64RMN6TP/C79988</t>
-  </si>
-  <si>
-    <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
-  </si>
-  <si>
-    <t>2Kb (256x8) I2C Serial EEPROM, 1.8-5.5V, SOIC-8</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>U202</t>
-  </si>
-  <si>
-    <t>SP330</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/MaxLinear-SP330EEY_LTR/C916084</t>
-  </si>
-  <si>
-    <t>TSSOP-24_4.4x7.8mm_P0.65mm</t>
-  </si>
-  <si>
-    <t>RS-232/RS-485/RS-422 Transceiver with 1.65V-5.5V Interface</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>U103</t>
-  </si>
-  <si>
-    <t>STM32G431RBTx</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/STMicroelectronics-STM32G431RBT6/C431633</t>
-  </si>
-  <si>
-    <t>LQFP-64_10x10mm_P0.5mm</t>
-  </si>
-  <si>
-    <t>STMicroelectronics Arm Cortex-M4 MCU, 128KB flash, 32KB RAM, 170 MHz, 1.71-3.6V, 52 GPIO, LQFP64</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>U401</t>
-  </si>
-  <si>
-    <t>TJA1042T</t>
-  </si>
-  <si>
-    <t>TJA1042T/1J</t>
-  </si>
-  <si>
-    <t>NXP Semicon</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/NXPSemicon-TJA1042T1J/C53670</t>
-  </si>
-  <si>
-    <t>High-Speed CAN Transceiver, standby mode, split pin, SOIC-8</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>U105 U303</t>
-  </si>
-  <si>
-    <t>USBLC6-2SC6</t>
-  </si>
-  <si>
-    <t>TECH PUBLIC</t>
-  </si>
-  <si>
-    <t>https://jlcpcb.com/partdetail/2790619-USBLC62SC6/C2687116</t>
-  </si>
-  <si>
-    <t>SOT-23-6</t>
-  </si>
-  <si>
-    <t>Very low capacitance ESD protection diode, 2 data-line, SOT-23-6</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>U301</t>
   </si>
   <si>
     <t>XC6206PxxxMR</t>
@@ -852,7 +852,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>3135853</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>48</xdr:row>
       <xdr:rowOff>173578</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1231,7 +1231,7 @@
         <v>219</v>
       </c>
       <c r="F3" s="3">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1245,7 +1245,7 @@
         <v>220</v>
       </c>
       <c r="F4" s="3">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1273,7 +1273,7 @@
         <v>222</v>
       </c>
       <c r="F6" s="3">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -1808,7 +1808,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="75" customHeight="1">
+    <row r="22" spans="1:12" ht="105" customHeight="1">
       <c r="A22" s="8" t="s">
         <v>109</v>
       </c>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ eurovibes/sertest-ng@5159d4b81fca0939de04461b6e2f5ac2f631fdfa 🚀
</commit_message>
<xml_diff>
--- a/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
+++ b/Fabrication/BoM/sertest-ng-bom_0.1.xlsx
@@ -350,7 +350,7 @@
     <t>14</t>
   </si>
   <si>
-    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R201 R202 R203 R204 R205 R206 R207 R208 R209 R210 R211 R212 R213 R214 R215 R216 R217 R218 R219 R220 R221 R222 R223 R224 R225 R226 R227 R228 R229 R230 R231 R232 R301 R302 R303 R401 R402 R403 R404</t>
+    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R201 R202 R203 R204 R205 R206 R207 R208 R209 R210 R211 R212 R213 R214 R215 R216 R217 R218 R219 R220 R221 R222 R223 R224 R225 R226 R227 R228 R229 R230 R231 R232 R301 R302 R303 R401 R402 R403 R404</t>
   </si>
   <si>
     <t>1 kΩ</t>
@@ -362,7 +362,7 @@
     <t>https://jlcpcb.com/partdetail/12256-0402WGF1001TCE/C11702 https://jlcpcb.com/partdetail/26648-0402WGF5101TCE/C25905 https://jlcpcb.com/partdetail/26826-0402WGF1004TCE/C26083 https://jlcpcb.com/partdetail/18646-1206W4F220JT5E/C17958 https://jlcpcb.com/partdetail/25848-0402WGF330JTCE/C25105 https://jlcpcb.com/partdetail/26487-0402WGF1002TCE/C25744 https://jlcpcb.com/partdetail/17853-0402WGF0000TCE/C17168</t>
   </si>
   <si>
-    <t>54</t>
+    <t>55</t>
   </si>
   <si>
     <t>15</t>
@@ -497,7 +497,7 @@
     <t>21</t>
   </si>
   <si>
-    <t>U101</t>
+    <t>U101 U106</t>
   </si>
   <si>
     <t>M24C02-RMN</t>
@@ -1231,7 +1231,7 @@
         <v>219</v>
       </c>
       <c r="F3" s="3">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1245,7 +1245,7 @@
         <v>220</v>
       </c>
       <c r="F4" s="3">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1273,7 +1273,7 @@
         <v>222</v>
       </c>
       <c r="F6" s="3">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2109,7 +2109,7 @@
         <v>164</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:12">

</xml_diff>